<commit_message>
improve descriptive and data cleaning scripts
</commit_message>
<xml_diff>
--- a/datasets/cleaned_response_dataset.xlsx
+++ b/datasets/cleaned_response_dataset.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Month</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>~2 Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>~2 Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2 Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Redmi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Honor</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Redmi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Msi (Laotop)</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4846,7 +4846,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Vivo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5494,7 +5494,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5782,7 +5782,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5854,7 +5854,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5926,7 +5926,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Vivo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5998,7 +5998,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6070,7 +6070,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6244,7 +6244,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6316,7 +6316,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6574,7 +6574,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6646,7 +6646,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6676,7 +6676,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -7222,7 +7222,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -7252,7 +7252,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -7324,7 +7324,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Redmi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -7396,7 +7396,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -7438,7 +7438,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -7540,7 +7540,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -7612,7 +7612,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -7684,7 +7684,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -7726,7 +7726,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -7798,7 +7798,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -7900,7 +7900,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -8116,7 +8116,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -8332,7 +8332,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -8374,7 +8374,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -8404,7 +8404,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -8446,7 +8446,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -8476,7 +8476,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -8590,7 +8590,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -8662,7 +8662,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -8692,7 +8692,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -8734,7 +8734,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -8806,7 +8806,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -8836,7 +8836,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -8878,7 +8878,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8950,7 +8950,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -8980,7 +8980,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -9052,7 +9052,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -9124,7 +9124,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -9166,7 +9166,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -9238,7 +9238,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -9268,7 +9268,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -9310,7 +9310,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -9340,7 +9340,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -9382,7 +9382,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -9412,7 +9412,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -9598,7 +9598,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Redmi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -9628,7 +9628,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -9700,7 +9700,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -9772,7 +9772,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -9886,7 +9886,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -9916,7 +9916,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -9988,7 +9988,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -10060,7 +10060,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -10102,7 +10102,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -10132,7 +10132,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -10174,7 +10174,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N136" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -10276,7 +10276,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -10318,7 +10318,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -10348,7 +10348,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -10420,7 +10420,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -10462,7 +10462,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -10534,7 +10534,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Huawei</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>I Didn'T Research Before Purchase</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -10636,7 +10636,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -10750,7 +10750,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -10780,7 +10780,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -10852,7 +10852,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -10894,7 +10894,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Asus</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -10966,7 +10966,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -11110,7 +11110,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -11212,7 +11212,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -11284,7 +11284,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>Only Few Hours</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -11326,7 +11326,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Msi</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -11428,7 +11428,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -11542,7 +11542,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Hp</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -11572,7 +11572,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -11758,7 +11758,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -11788,7 +11788,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>Few Weeks</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>Few Months</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>Only Few Days</t>
+          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">

</xml_diff>

<commit_message>
bug_fix: missing parenthesis when calling title() when standardizing column names
</commit_message>
<xml_diff>
--- a/datasets/cleaned_response_dataset.xlsx
+++ b/datasets/cleaned_response_dataset.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Redmi</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Honor</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Redmi</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi (Laotop)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4846,7 +4846,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Vivo</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5494,7 +5494,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5782,7 +5782,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5854,7 +5854,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5926,7 +5926,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Vivo</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5998,7 +5998,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6070,7 +6070,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6244,7 +6244,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6316,7 +6316,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6574,7 +6574,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6646,7 +6646,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6676,7 +6676,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -7222,7 +7222,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -7252,7 +7252,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -7324,7 +7324,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Redmi</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -7396,7 +7396,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -7438,7 +7438,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -7540,7 +7540,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -7612,7 +7612,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -7684,7 +7684,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -7726,7 +7726,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -7798,7 +7798,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -7900,7 +7900,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -8116,7 +8116,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -8332,7 +8332,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -8374,7 +8374,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -8404,7 +8404,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -8446,7 +8446,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -8476,7 +8476,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -8590,7 +8590,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -8662,7 +8662,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -8692,7 +8692,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -8734,7 +8734,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -8806,7 +8806,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -8836,7 +8836,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -8878,7 +8878,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8950,7 +8950,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -8980,7 +8980,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -9052,7 +9052,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -9124,7 +9124,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -9166,7 +9166,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -9238,7 +9238,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -9268,7 +9268,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -9310,7 +9310,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -9340,7 +9340,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -9382,7 +9382,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -9412,7 +9412,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -9598,7 +9598,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Redmi</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -9628,7 +9628,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -9700,7 +9700,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -9772,7 +9772,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -9886,7 +9886,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -9916,7 +9916,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -9988,7 +9988,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -10060,7 +10060,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -10102,7 +10102,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -10132,7 +10132,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -10174,7 +10174,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N136" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -10276,7 +10276,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -10318,7 +10318,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -10348,7 +10348,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -10420,7 +10420,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -10462,7 +10462,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -10534,7 +10534,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Huawei</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -10636,7 +10636,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -10750,7 +10750,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -10780,7 +10780,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -10852,7 +10852,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -10894,7 +10894,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Asus</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -10966,7 +10966,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -11110,7 +11110,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -11212,7 +11212,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -11284,7 +11284,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -11326,7 +11326,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -11428,7 +11428,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -11542,7 +11542,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Hp</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -11572,7 +11572,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -11758,7 +11758,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -11788,7 +11788,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20548d20d0&gt;&gt;</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>&lt;bound method StringMethods.title of &lt;pandas.core.strings.accessor.StringMethods object at 0x7f20546b51d0&gt;&gt;</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">

</xml_diff>